<commit_message>
Bump to net8.0, add docs and config updates
Upgrade project target framework to .NET 8.0 and add XML documentation across core types (DeviceMetaData, CommandClassifier, Logger, MeterClientsGenerator, MeterConfiguration, MeterConfigurationUI). Introduce DeviceMetaData helpers (PerformCommand, GetDataCommand) and MeterConfiguration save/load helpers. Surface configuration fields and SetupGlobalConfiguration in MeterClientsGenerator, and document async networking helpers (ReadCommand, SendCommandAsync, ProcessCommandAsync) in the UI. Update appsettings defaults to localhost, port, file paths and database connection string, and replace the Excel source file (meter1.xlsx). These changes improve code readability, provide basic API docs, and adjust runtime/config defaults for local testing.
</commit_message>
<xml_diff>
--- a/MeterClient/meter1.xlsx
+++ b/MeterClient/meter1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Umair\Documents\Repositories\Meter\MeterClient\MeterClient\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robass Atif\Desktop\mdc\MeterClient\MeterClient\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1237ECBB-A334-4E41-B5C7-C783DC69DCC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28BDF43C-25E7-4711-A221-C6CB360E6EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -383,10 +383,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C25000"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -405,7 +405,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>3098001001</v>
+        <v>3097000001</v>
       </c>
       <c r="C2" s="1">
         <v>12345678</v>
@@ -511,1026 +511,306 @@
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>3098001011</v>
-      </c>
-      <c r="C12" s="1">
-        <v>12345678</v>
-      </c>
+      <c r="C12" s="1"/>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>3098001012</v>
-      </c>
-      <c r="C13" s="1">
-        <v>12345678</v>
-      </c>
+      <c r="C13" s="1"/>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>3098001013</v>
-      </c>
-      <c r="C14" s="1">
-        <v>12345678</v>
-      </c>
+      <c r="C14" s="1"/>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>3098001014</v>
-      </c>
-      <c r="C15" s="1">
-        <v>12345678</v>
-      </c>
+      <c r="C15" s="1"/>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>3098001015</v>
-      </c>
-      <c r="C16" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>3098001016</v>
-      </c>
-      <c r="C17" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18">
-        <v>3098001017</v>
-      </c>
-      <c r="C18" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19">
-        <v>3098001018</v>
-      </c>
-      <c r="C19" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>3098001019</v>
-      </c>
-      <c r="C20" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>3098001020</v>
-      </c>
-      <c r="C21" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22">
-        <v>3098001021</v>
-      </c>
-      <c r="C22" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23">
-        <v>3098001022</v>
-      </c>
-      <c r="C23" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24">
-        <v>3098001023</v>
-      </c>
-      <c r="C24" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>3098001024</v>
-      </c>
-      <c r="C25" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26">
-        <v>3098001025</v>
-      </c>
-      <c r="C26" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27">
-        <v>3098001026</v>
-      </c>
-      <c r="C27" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28">
-        <v>3098001027</v>
-      </c>
-      <c r="C28" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29">
-        <v>3098001028</v>
-      </c>
-      <c r="C29" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30">
-        <v>3098001029</v>
-      </c>
-      <c r="C30" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31">
-        <v>3098001030</v>
-      </c>
-      <c r="C31" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32">
-        <v>3098001031</v>
-      </c>
-      <c r="C32" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33">
-        <v>3098001032</v>
-      </c>
-      <c r="C33" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34">
-        <v>33</v>
-      </c>
-      <c r="B34">
-        <v>3098001033</v>
-      </c>
-      <c r="C34" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35">
-        <v>3098001034</v>
-      </c>
-      <c r="C35" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36">
-        <v>3098001035</v>
-      </c>
-      <c r="C36" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37">
-        <v>3098001036</v>
-      </c>
-      <c r="C37" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38">
-        <v>37</v>
-      </c>
-      <c r="B38">
-        <v>3098001037</v>
-      </c>
-      <c r="C38" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39">
-        <v>3098001038</v>
-      </c>
-      <c r="C39" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40">
-        <v>3098001039</v>
-      </c>
-      <c r="C40" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41">
-        <v>3098001040</v>
-      </c>
-      <c r="C41" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42">
-        <v>3098001041</v>
-      </c>
-      <c r="C42" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43">
-        <v>3098001042</v>
-      </c>
-      <c r="C43" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44">
-        <v>3098001043</v>
-      </c>
-      <c r="C44" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45">
-        <v>44</v>
-      </c>
-      <c r="B45">
-        <v>3098001044</v>
-      </c>
-      <c r="C45" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46">
-        <v>45</v>
-      </c>
-      <c r="B46">
-        <v>3098001045</v>
-      </c>
-      <c r="C46" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47">
-        <v>46</v>
-      </c>
-      <c r="B47">
-        <v>3098001046</v>
-      </c>
-      <c r="C47" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48">
-        <v>47</v>
-      </c>
-      <c r="B48">
-        <v>3098001047</v>
-      </c>
-      <c r="C48" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49">
-        <v>48</v>
-      </c>
-      <c r="B49">
-        <v>3098001048</v>
-      </c>
-      <c r="C49" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="A50">
-        <v>49</v>
-      </c>
-      <c r="B50">
-        <v>3098001049</v>
-      </c>
-      <c r="C50" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3">
-      <c r="A51">
-        <v>50</v>
-      </c>
-      <c r="B51">
-        <v>3098001050</v>
-      </c>
-      <c r="C51" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52">
-        <v>51</v>
-      </c>
-      <c r="B52">
-        <v>3098001051</v>
-      </c>
-      <c r="C52" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53">
-        <v>52</v>
-      </c>
-      <c r="B53">
-        <v>3098001052</v>
-      </c>
-      <c r="C53" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54">
-        <v>53</v>
-      </c>
-      <c r="B54">
-        <v>3098001053</v>
-      </c>
-      <c r="C54" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55">
-        <v>54</v>
-      </c>
-      <c r="B55">
-        <v>3098001054</v>
-      </c>
-      <c r="C55" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="A56">
-        <v>55</v>
-      </c>
-      <c r="B56">
-        <v>3098001055</v>
-      </c>
-      <c r="C56" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="A57">
-        <v>56</v>
-      </c>
-      <c r="B57">
-        <v>3098001056</v>
-      </c>
-      <c r="C57" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58">
-        <v>57</v>
-      </c>
-      <c r="B58">
-        <v>3098001057</v>
-      </c>
-      <c r="C58" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3">
-      <c r="A59">
-        <v>58</v>
-      </c>
-      <c r="B59">
-        <v>3098001058</v>
-      </c>
-      <c r="C59" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3">
-      <c r="A60">
-        <v>59</v>
-      </c>
-      <c r="B60">
-        <v>3098001059</v>
-      </c>
-      <c r="C60" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3">
-      <c r="A61">
-        <v>60</v>
-      </c>
-      <c r="B61">
-        <v>3098001060</v>
-      </c>
-      <c r="C61" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3">
-      <c r="A62">
-        <v>61</v>
-      </c>
-      <c r="B62">
-        <v>3098001061</v>
-      </c>
-      <c r="C62" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63">
-        <v>62</v>
-      </c>
-      <c r="B63">
-        <v>3098001062</v>
-      </c>
-      <c r="C63" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3">
-      <c r="A64">
-        <v>63</v>
-      </c>
-      <c r="B64">
-        <v>3098001063</v>
-      </c>
-      <c r="C64" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3">
-      <c r="A65">
-        <v>64</v>
-      </c>
-      <c r="B65">
-        <v>3098001064</v>
-      </c>
-      <c r="C65" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3">
-      <c r="A66">
-        <v>65</v>
-      </c>
-      <c r="B66">
-        <v>3098001065</v>
-      </c>
-      <c r="C66" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3">
-      <c r="A67">
-        <v>66</v>
-      </c>
-      <c r="B67">
-        <v>3098001066</v>
-      </c>
-      <c r="C67" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3">
-      <c r="A68">
-        <v>67</v>
-      </c>
-      <c r="B68">
-        <v>3098001067</v>
-      </c>
-      <c r="C68" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3">
-      <c r="A69">
-        <v>68</v>
-      </c>
-      <c r="B69">
-        <v>3098001068</v>
-      </c>
-      <c r="C69" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3">
-      <c r="A70">
-        <v>69</v>
-      </c>
-      <c r="B70">
-        <v>3098001069</v>
-      </c>
-      <c r="C70" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3">
-      <c r="A71">
-        <v>70</v>
-      </c>
-      <c r="B71">
-        <v>3098001070</v>
-      </c>
-      <c r="C71" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3">
-      <c r="A72">
-        <v>71</v>
-      </c>
-      <c r="B72">
-        <v>3098001071</v>
-      </c>
-      <c r="C72" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3">
-      <c r="A73">
-        <v>72</v>
-      </c>
-      <c r="B73">
-        <v>3098001072</v>
-      </c>
-      <c r="C73" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3">
-      <c r="A74">
-        <v>73</v>
-      </c>
-      <c r="B74">
-        <v>3098001073</v>
-      </c>
-      <c r="C74" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3">
-      <c r="A75">
-        <v>74</v>
-      </c>
-      <c r="B75">
-        <v>3098001074</v>
-      </c>
-      <c r="C75" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3">
-      <c r="A76">
-        <v>75</v>
-      </c>
-      <c r="B76">
-        <v>3098001075</v>
-      </c>
-      <c r="C76" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3">
-      <c r="A77">
-        <v>76</v>
-      </c>
-      <c r="B77">
-        <v>3098001076</v>
-      </c>
-      <c r="C77" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3">
-      <c r="A78">
-        <v>77</v>
-      </c>
-      <c r="B78">
-        <v>3098001077</v>
-      </c>
-      <c r="C78" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3">
-      <c r="A79">
-        <v>78</v>
-      </c>
-      <c r="B79">
-        <v>3098001078</v>
-      </c>
-      <c r="C79" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3">
-      <c r="A80">
-        <v>79</v>
-      </c>
-      <c r="B80">
-        <v>3098001079</v>
-      </c>
-      <c r="C80" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3">
-      <c r="A81">
-        <v>80</v>
-      </c>
-      <c r="B81">
-        <v>3098001080</v>
-      </c>
-      <c r="C81" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3">
-      <c r="A82">
-        <v>81</v>
-      </c>
-      <c r="B82">
-        <v>3098001081</v>
-      </c>
-      <c r="C82" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3">
-      <c r="A83">
-        <v>82</v>
-      </c>
-      <c r="B83">
-        <v>3098001082</v>
-      </c>
-      <c r="C83" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3">
-      <c r="A84">
-        <v>83</v>
-      </c>
-      <c r="B84">
-        <v>3098001083</v>
-      </c>
-      <c r="C84" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3">
-      <c r="A85">
-        <v>84</v>
-      </c>
-      <c r="B85">
-        <v>3098001084</v>
-      </c>
-      <c r="C85" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3">
-      <c r="A86">
-        <v>85</v>
-      </c>
-      <c r="B86">
-        <v>3098001085</v>
-      </c>
-      <c r="C86" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3">
-      <c r="A87">
-        <v>86</v>
-      </c>
-      <c r="B87">
-        <v>3098001086</v>
-      </c>
-      <c r="C87" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3">
-      <c r="A88">
-        <v>87</v>
-      </c>
-      <c r="B88">
-        <v>3098001087</v>
-      </c>
-      <c r="C88" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3">
-      <c r="A89">
-        <v>88</v>
-      </c>
-      <c r="B89">
-        <v>3098001088</v>
-      </c>
-      <c r="C89" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3">
-      <c r="A90">
-        <v>89</v>
-      </c>
-      <c r="B90">
-        <v>3098001089</v>
-      </c>
-      <c r="C90" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3">
-      <c r="A91">
-        <v>90</v>
-      </c>
-      <c r="B91">
-        <v>3098001090</v>
-      </c>
-      <c r="C91" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3">
-      <c r="A92">
-        <v>91</v>
-      </c>
-      <c r="B92">
-        <v>3098001091</v>
-      </c>
-      <c r="C92" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3">
-      <c r="A93">
-        <v>92</v>
-      </c>
-      <c r="B93">
-        <v>3098001092</v>
-      </c>
-      <c r="C93" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3">
-      <c r="A94">
-        <v>93</v>
-      </c>
-      <c r="B94">
-        <v>3098001093</v>
-      </c>
-      <c r="C94" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3">
-      <c r="A95">
-        <v>94</v>
-      </c>
-      <c r="B95">
-        <v>3098001094</v>
-      </c>
-      <c r="C95" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3">
-      <c r="A96">
-        <v>95</v>
-      </c>
-      <c r="B96">
-        <v>3098001095</v>
-      </c>
-      <c r="C96" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3">
-      <c r="A97">
-        <v>96</v>
-      </c>
-      <c r="B97">
-        <v>3098001096</v>
-      </c>
-      <c r="C97" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3">
-      <c r="A98">
-        <v>97</v>
-      </c>
-      <c r="B98">
-        <v>3098001097</v>
-      </c>
-      <c r="C98" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3">
-      <c r="A99">
-        <v>98</v>
-      </c>
-      <c r="B99">
-        <v>3098001098</v>
-      </c>
-      <c r="C99" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3">
-      <c r="A100">
-        <v>99</v>
-      </c>
-      <c r="B100">
-        <v>3098001099</v>
-      </c>
-      <c r="C100" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3">
-      <c r="A101">
-        <v>100</v>
-      </c>
-      <c r="B101">
-        <v>3098001100</v>
-      </c>
-      <c r="C101" s="1">
-        <v>12345678</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3">
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" s="1"/>
+    </row>
+    <row r="18" spans="3:3">
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" spans="3:3">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="3:3">
+      <c r="C20" s="1"/>
+    </row>
+    <row r="21" spans="3:3">
+      <c r="C21" s="1"/>
+    </row>
+    <row r="22" spans="3:3">
+      <c r="C22" s="1"/>
+    </row>
+    <row r="23" spans="3:3">
+      <c r="C23" s="1"/>
+    </row>
+    <row r="24" spans="3:3">
+      <c r="C24" s="1"/>
+    </row>
+    <row r="25" spans="3:3">
+      <c r="C25" s="1"/>
+    </row>
+    <row r="26" spans="3:3">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="3:3">
+      <c r="C27" s="1"/>
+    </row>
+    <row r="28" spans="3:3">
+      <c r="C28" s="1"/>
+    </row>
+    <row r="29" spans="3:3">
+      <c r="C29" s="1"/>
+    </row>
+    <row r="30" spans="3:3">
+      <c r="C30" s="1"/>
+    </row>
+    <row r="31" spans="3:3">
+      <c r="C31" s="1"/>
+    </row>
+    <row r="32" spans="3:3">
+      <c r="C32" s="1"/>
+    </row>
+    <row r="33" spans="3:3">
+      <c r="C33" s="1"/>
+    </row>
+    <row r="34" spans="3:3">
+      <c r="C34" s="1"/>
+    </row>
+    <row r="35" spans="3:3">
+      <c r="C35" s="1"/>
+    </row>
+    <row r="36" spans="3:3">
+      <c r="C36" s="1"/>
+    </row>
+    <row r="37" spans="3:3">
+      <c r="C37" s="1"/>
+    </row>
+    <row r="38" spans="3:3">
+      <c r="C38" s="1"/>
+    </row>
+    <row r="39" spans="3:3">
+      <c r="C39" s="1"/>
+    </row>
+    <row r="40" spans="3:3">
+      <c r="C40" s="1"/>
+    </row>
+    <row r="41" spans="3:3">
+      <c r="C41" s="1"/>
+    </row>
+    <row r="42" spans="3:3">
+      <c r="C42" s="1"/>
+    </row>
+    <row r="43" spans="3:3">
+      <c r="C43" s="1"/>
+    </row>
+    <row r="44" spans="3:3">
+      <c r="C44" s="1"/>
+    </row>
+    <row r="45" spans="3:3">
+      <c r="C45" s="1"/>
+    </row>
+    <row r="46" spans="3:3">
+      <c r="C46" s="1"/>
+    </row>
+    <row r="47" spans="3:3">
+      <c r="C47" s="1"/>
+    </row>
+    <row r="48" spans="3:3">
+      <c r="C48" s="1"/>
+    </row>
+    <row r="49" spans="3:3">
+      <c r="C49" s="1"/>
+    </row>
+    <row r="50" spans="3:3">
+      <c r="C50" s="1"/>
+    </row>
+    <row r="51" spans="3:3">
+      <c r="C51" s="1"/>
+    </row>
+    <row r="52" spans="3:3">
+      <c r="C52" s="1"/>
+    </row>
+    <row r="53" spans="3:3">
+      <c r="C53" s="1"/>
+    </row>
+    <row r="54" spans="3:3">
+      <c r="C54" s="1"/>
+    </row>
+    <row r="55" spans="3:3">
+      <c r="C55" s="1"/>
+    </row>
+    <row r="56" spans="3:3">
+      <c r="C56" s="1"/>
+    </row>
+    <row r="57" spans="3:3">
+      <c r="C57" s="1"/>
+    </row>
+    <row r="58" spans="3:3">
+      <c r="C58" s="1"/>
+    </row>
+    <row r="59" spans="3:3">
+      <c r="C59" s="1"/>
+    </row>
+    <row r="60" spans="3:3">
+      <c r="C60" s="1"/>
+    </row>
+    <row r="61" spans="3:3">
+      <c r="C61" s="1"/>
+    </row>
+    <row r="62" spans="3:3">
+      <c r="C62" s="1"/>
+    </row>
+    <row r="63" spans="3:3">
+      <c r="C63" s="1"/>
+    </row>
+    <row r="64" spans="3:3">
+      <c r="C64" s="1"/>
+    </row>
+    <row r="65" spans="3:3">
+      <c r="C65" s="1"/>
+    </row>
+    <row r="66" spans="3:3">
+      <c r="C66" s="1"/>
+    </row>
+    <row r="67" spans="3:3">
+      <c r="C67" s="1"/>
+    </row>
+    <row r="68" spans="3:3">
+      <c r="C68" s="1"/>
+    </row>
+    <row r="69" spans="3:3">
+      <c r="C69" s="1"/>
+    </row>
+    <row r="70" spans="3:3">
+      <c r="C70" s="1"/>
+    </row>
+    <row r="71" spans="3:3">
+      <c r="C71" s="1"/>
+    </row>
+    <row r="72" spans="3:3">
+      <c r="C72" s="1"/>
+    </row>
+    <row r="73" spans="3:3">
+      <c r="C73" s="1"/>
+    </row>
+    <row r="74" spans="3:3">
+      <c r="C74" s="1"/>
+    </row>
+    <row r="75" spans="3:3">
+      <c r="C75" s="1"/>
+    </row>
+    <row r="76" spans="3:3">
+      <c r="C76" s="1"/>
+    </row>
+    <row r="77" spans="3:3">
+      <c r="C77" s="1"/>
+    </row>
+    <row r="78" spans="3:3">
+      <c r="C78" s="1"/>
+    </row>
+    <row r="79" spans="3:3">
+      <c r="C79" s="1"/>
+    </row>
+    <row r="80" spans="3:3">
+      <c r="C80" s="1"/>
+    </row>
+    <row r="81" spans="3:3">
+      <c r="C81" s="1"/>
+    </row>
+    <row r="82" spans="3:3">
+      <c r="C82" s="1"/>
+    </row>
+    <row r="83" spans="3:3">
+      <c r="C83" s="1"/>
+    </row>
+    <row r="84" spans="3:3">
+      <c r="C84" s="1"/>
+    </row>
+    <row r="85" spans="3:3">
+      <c r="C85" s="1"/>
+    </row>
+    <row r="86" spans="3:3">
+      <c r="C86" s="1"/>
+    </row>
+    <row r="87" spans="3:3">
+      <c r="C87" s="1"/>
+    </row>
+    <row r="88" spans="3:3">
+      <c r="C88" s="1"/>
+    </row>
+    <row r="89" spans="3:3">
+      <c r="C89" s="1"/>
+    </row>
+    <row r="90" spans="3:3">
+      <c r="C90" s="1"/>
+    </row>
+    <row r="91" spans="3:3">
+      <c r="C91" s="1"/>
+    </row>
+    <row r="92" spans="3:3">
+      <c r="C92" s="1"/>
+    </row>
+    <row r="93" spans="3:3">
+      <c r="C93" s="1"/>
+    </row>
+    <row r="94" spans="3:3">
+      <c r="C94" s="1"/>
+    </row>
+    <row r="95" spans="3:3">
+      <c r="C95" s="1"/>
+    </row>
+    <row r="96" spans="3:3">
+      <c r="C96" s="1"/>
+    </row>
+    <row r="97" spans="3:3">
+      <c r="C97" s="1"/>
+    </row>
+    <row r="98" spans="3:3">
+      <c r="C98" s="1"/>
+    </row>
+    <row r="99" spans="3:3">
+      <c r="C99" s="1"/>
+    </row>
+    <row r="100" spans="3:3">
+      <c r="C100" s="1"/>
+    </row>
+    <row r="101" spans="3:3">
+      <c r="C101" s="1"/>
+    </row>
+    <row r="102" spans="3:3">
       <c r="C102" s="1"/>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="3:3">
       <c r="C103" s="1"/>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="3:3">
       <c r="C104" s="1"/>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="3:3">
       <c r="C105" s="1"/>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="3:3">
       <c r="C106" s="1"/>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="3:3">
       <c r="C107" s="1"/>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="3:3">
       <c r="C108" s="1"/>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="3:3">
       <c r="C109" s="1"/>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="3:3">
       <c r="C110" s="1"/>
     </row>
-    <row r="111" spans="1:3">
+    <row r="111" spans="3:3">
       <c r="C111" s="1"/>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="3:3">
       <c r="C112" s="1"/>
     </row>
     <row r="113" spans="3:3">

</xml_diff>